<commit_message>
feat: add blocked_word table for chat filtering and name validation
- Add blocked_word table with src/dst fields for word replacement
- Implement contains_substring method for name validation
- Implement filter method for chat message filtering
- Add blocked_word validation to login server (after blocked_name check)
- Apply chat message filtering in game server chat handler
- Add extension methods to both login and game model.additional.h
</commit_message>
<xml_diff>
--- a/resources/table/blocked.xlsx
+++ b/resources/table/blocked.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D714F305-502C-4ABB-AC66-6FF83DE6E6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E30243-E8BF-4533-8908-289CF7B8739F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="blocked_name" sheetId="1" r:id="rId1"/>
+    <sheet name="blocked_word" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>server</t>
   </si>
@@ -42,6 +43,38 @@
   </si>
   <si>
     <t>관리자</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>server</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>src</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dst</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>string</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>꺼져</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>가세요</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>씨발</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>어머</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -96,11 +129,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -464,4 +500,58 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD87A90A-3873-4FC4-88E4-A94333B47DA8}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>